<commit_message>
feat: Implement 'Ajuste y Cuadre de Camas' dual-panel workspace, block division modal, spray lance tracking, and printable order enhancements
</commit_message>
<xml_diff>
--- a/productos y dosis.xlsx
+++ b/productos y dosis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\todo en vs code\fumigacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C704B28B-D691-4675-A9EB-6A57D58D650B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE9CC23A-71C0-4FEE-B698-6D3199A957DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{4CA33D79-6991-4A2D-B868-16E7753E449D}"/>
   </bookViews>
@@ -3587,6 +3587,7 @@
     <col min="2" max="2" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="29.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="58.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>